<commit_message>
Updated delstandardization github link.
</commit_message>
<xml_diff>
--- a/www/sosdar-StatsInExcel-DELsTAndardization.xlsx
+++ b/www/sosdar-StatsInExcel-DELsTAndardization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sosda\workspace\StatsInExcel\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE4E75D-1099-4940-9AFE-27028CCFC782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD6085F5-73C5-4006-BFAD-2C6FAAA93612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="4" xr2:uid="{B33C48E6-AC3F-4551-954B-29E644381288}"/>
   </bookViews>
@@ -479,7 +479,7 @@
     <t>D</t>
   </si>
   <si>
-    <t>https://github.com/sosdar2025/StatsInExcel/blob/main/www/sosdar-StatsInExcel-DELsTAndardization.xls</t>
+    <t>https://github.com/sosdar2025/StatsInExcel/blob/main/www/sosdar-StatsInExcel-DELsTAndardization.xlsx</t>
   </si>
 </sst>
 </file>
@@ -12985,7 +12985,7 @@
       <c r="E1970" s="56"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="PUkxWOuRjUZD1/O4/oHsmcOrSZFo/lAh6jc+K4nt91Q7Js8Z8XZFSN1+tvd4is1XZ4FzECEGU6EifiQ25NHdUw==" saltValue="29dqoMbyag17SbtbWfQ0aQ==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="0INwIy/ahUBtbJrpb6sZB+hOsNH4sxjDXgxXZFVmr9ExJEvsgVTRYWo6sAhnerOLjm1lb5LfJhQpGXxYkd+Avw==" saltValue="/UXjsufwW894G757tUYSkQ==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" xr:uid="{A7009A2D-26FF-47DD-9178-7782A74F75B6}"/>
     <hyperlink ref="E3" r:id="rId2" xr:uid="{C0C89D26-1655-4DD3-BD3F-64E2305FAD7F}"/>
@@ -13068,19 +13068,19 @@
       </c>
       <c r="B7" s="46">
         <f t="shared" ref="B7:G7" ca="1" si="0">AVERAGE(B11:B1010)</f>
-        <v>174.37254151617799</v>
+        <v>182.74181337304236</v>
       </c>
       <c r="C7" s="45">
         <f t="shared" ca="1" si="0"/>
-        <v>174.37254151617799</v>
+        <v>182.74181337304236</v>
       </c>
       <c r="D7" s="45">
         <f t="shared" ca="1" si="0"/>
-        <v>2.1384413016303783E-3</v>
+        <v>9.1792566005444165E-6</v>
       </c>
       <c r="E7" s="46">
         <f t="shared" ca="1" si="0"/>
-        <v>174.74542696082642</v>
+        <v>182.74349080703897</v>
       </c>
       <c r="F7" s="45">
         <f t="shared" ca="1" si="0"/>
@@ -13088,7 +13088,7 @@
       </c>
       <c r="G7" s="45">
         <f t="shared" ca="1" si="0"/>
-        <v>-1.7763568394002505E-15</v>
+        <v>2.5701663020072374E-14</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -13097,27 +13097,27 @@
       </c>
       <c r="B8" s="47">
         <f t="shared" ref="B8:G8" ca="1" si="1">STDEV(B11:B1010)</f>
-        <v>8.059251525734588</v>
+        <v>0.55365686436587958</v>
       </c>
       <c r="C8" s="45">
         <f t="shared" ca="1" si="1"/>
-        <v>8.059251525734588</v>
+        <v>0.55365686436587958</v>
       </c>
       <c r="D8" s="48">
         <f t="shared" ca="1" si="1"/>
-        <v>9.2535998773035019E-2</v>
+        <v>6.0594715049136433E-3</v>
       </c>
       <c r="E8" s="47">
         <f t="shared" ca="1" si="1"/>
-        <v>16.13573728779205</v>
+        <v>1.1073188108901915</v>
       </c>
       <c r="F8" s="45">
         <f t="shared" ca="1" si="1"/>
-        <v>0.99999999999999989</v>
+        <v>1</v>
       </c>
       <c r="G8" s="45">
         <f t="shared" ca="1" si="1"/>
-        <v>0.99999999999999989</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -13155,27 +13155,27 @@
       </c>
       <c r="B11" s="50">
         <f ca="1">IF(ISNUMBER(A11),_xlfn.NORM.INV(RAND(),$B$2,$B$3),"")</f>
-        <v>168.67379011104302</v>
+        <v>182.35031884979878</v>
       </c>
       <c r="C11" s="50">
         <f ca="1">IF(ISNUMBER(B11),(SUM($B$11:$B$1010)-B11)/($B$4-1),"")</f>
-        <v>180.07129292131296</v>
+        <v>183.13330789628594</v>
       </c>
       <c r="D11" s="45">
         <f t="shared" ref="D11:D74" ca="1" si="2">IF(ISNUMBER(B11),(($B$4-1)*B11/(SUM($B$11:$B$1010)-B11)-1),"")</f>
-        <v>-6.3294390934652722E-2</v>
+        <v>-4.275514134930547E-3</v>
       </c>
       <c r="E11" s="50">
         <f t="shared" ref="E11:E74" ca="1" si="3">IF(ISNUMBER(B11),AVERAGE($B$11:$B$1010)*(1+D11),"")</f>
-        <v>163.33573770518404</v>
+        <v>181.96049816692309</v>
       </c>
       <c r="F11" s="45">
         <f t="shared" ref="F11:F74" ca="1" si="4">IF(ISNUMBER(D11),(D11-AVERAGE($D$11:$D$1010))/STDEV($D$11:$D$1010),"")</f>
-        <v>-0.70710678118654746</v>
+        <v>-0.70710678118654757</v>
       </c>
       <c r="G11" s="45">
         <f t="shared" ref="G11:G74" ca="1" si="5">IF(ISNUMBER(B11),(B11-AVERAGE($B$11:$B$20))/STDEV($B$11:$B$20),"")</f>
-        <v>-0.70710678118654924</v>
+        <v>-0.70710678118652182</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -13185,27 +13185,27 @@
       </c>
       <c r="B12" s="50">
         <f t="shared" ref="B12:B75" ca="1" si="6">IF(ISNUMBER(A12),_xlfn.NORM.INV(RAND(),$B$2,$B$3),"")</f>
-        <v>180.07129292131293</v>
+        <v>183.13330789628597</v>
       </c>
       <c r="C12" s="50">
         <f t="shared" ref="C12:C75" ca="1" si="7">IF(ISNUMBER(B12),(SUM($B$11:$B$1010)-B12)/($B$4-1),"")</f>
-        <v>168.67379011104305</v>
+        <v>182.35031884979875</v>
       </c>
       <c r="D12" s="45">
         <f t="shared" ca="1" si="2"/>
-        <v>6.7571273537913479E-2</v>
+        <v>4.2938726481316358E-3</v>
       </c>
       <c r="E12" s="50">
         <f t="shared" ca="1" si="3"/>
-        <v>186.15511621646883</v>
+        <v>183.52648344715485</v>
       </c>
       <c r="F12" s="45">
         <f t="shared" ca="1" si="4"/>
-        <v>0.70710678118654746</v>
+        <v>0.70710678118654757</v>
       </c>
       <c r="G12" s="45">
         <f t="shared" ca="1" si="5"/>
-        <v>0.70710678118654569</v>
+        <v>0.70710678118657322</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
@@ -46088,26 +46088,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="297242e2-fbb8-4c67-99ce-cd3528d8cbc6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2b487279-c3ab-426b-b6cf-53277d34fdd2" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100956A0F4035FD3E439A1375AA81288D3D" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="629d0db9554db0b6d69858e5d10e2081">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="297242e2-fbb8-4c67-99ce-cd3528d8cbc6" xmlns:ns3="2b487279-c3ab-426b-b6cf-53277d34fdd2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="10effca0874d89e46752f2faf5212ccb" ns2:_="" ns3:_="">
     <xsd:import namespace="297242e2-fbb8-4c67-99ce-cd3528d8cbc6"/>
@@ -46330,10 +46310,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="297242e2-fbb8-4c67-99ce-cd3528d8cbc6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2b487279-c3ab-426b-b6cf-53277d34fdd2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D65EDFB4-7AB7-4358-93FB-FC0B1840C267}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6277D62E-5E45-4A72-AFF1-71084806AE04}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="297242e2-fbb8-4c67-99ce-cd3528d8cbc6"/>
+    <ds:schemaRef ds:uri="2b487279-c3ab-426b-b6cf-53277d34fdd2"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -46350,20 +46361,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6277D62E-5E45-4A72-AFF1-71084806AE04}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D65EDFB4-7AB7-4358-93FB-FC0B1840C267}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="297242e2-fbb8-4c67-99ce-cd3528d8cbc6"/>
-    <ds:schemaRef ds:uri="2b487279-c3ab-426b-b6cf-53277d34fdd2"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated DELsTAndardization file after publishing video.
</commit_message>
<xml_diff>
--- a/www/sosdar-StatsInExcel-DELsTAndardization.xlsx
+++ b/www/sosdar-StatsInExcel-DELsTAndardization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sosda\workspace\StatsInExcel\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E61D424-228D-49E2-85E7-BC9FDD8DCA5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CC32A4F-5E63-4F85-A434-2F525128FC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="4" xr2:uid="{B33C48E6-AC3F-4551-954B-29E644381288}"/>
   </bookViews>
@@ -473,13 +473,13 @@
     <t>sosdar2025@outlook.com</t>
   </si>
   <si>
-    <t>https://youtu.be/o6-8Fpar9os</t>
-  </si>
-  <si>
     <t>D</t>
   </si>
   <si>
     <t>https://github.com/sosdar2025/StatsInExcel/blob/main/www/sosdar-StatsInExcel-DELsTAndardization.xlsx</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Lo9kDBaZeV4</t>
   </si>
 </sst>
 </file>
@@ -490,7 +490,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -571,13 +571,6 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="0"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -804,7 +797,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -886,8 +879,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="3" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="4" applyFill="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="2" applyFill="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="5" applyFont="1" applyFill="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1023,6 +1015,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="5" name="Picture 4">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{74DBB8E6-97AD-EB32-E64D-F1300D6651C6}"/>
@@ -1034,7 +1027,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -1084,7 +1077,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -13012,24 +13005,24 @@
     </row>
     <row r="3" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E3" s="54" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E4" s="54" t="s">
         <v>117</v>
-      </c>
-    </row>
-    <row r="4" spans="5:5" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="E4" s="55" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="1000" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E1000" s="52" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="1970" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E1970" s="56"/>
+      <c r="E1970" s="55"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="0INwIy/ahUBtbJrpb6sZB+hOsNH4sxjDXgxXZFVmr9ExJEvsgVTRYWo6sAhnerOLjm1lb5LfJhQpGXxYkd+Avw==" saltValue="/UXjsufwW894G757tUYSkQ==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="qCW7GF7SlhAI+JOjYpcQ50Q+h0dfFZhv53gY3suM8nS1hr7XHJ5t6FBoeDKWgzp9wJvaI5q0t4gGZfbV4J3zRw==" saltValue="WBEC/gO2V5ycGuak/AwcBg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" xr:uid="{A7009A2D-26FF-47DD-9178-7782A74F75B6}"/>
     <hyperlink ref="E3" r:id="rId2" xr:uid="{C0C89D26-1655-4DD3-BD3F-64E2305FAD7F}"/>
@@ -13052,16 +13045,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="56" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="39" t="s">
@@ -13112,19 +13105,19 @@
       </c>
       <c r="B7" s="46">
         <f t="shared" ref="B7:G7" ca="1" si="0">AVERAGE(B11:B1010)</f>
-        <v>171.91238971205823</v>
+        <v>172.74279683894378</v>
       </c>
       <c r="C7" s="45">
         <f t="shared" ca="1" si="0"/>
-        <v>171.91238971205823</v>
+        <v>172.74279683894378</v>
       </c>
       <c r="D7" s="45">
         <f t="shared" ca="1" si="0"/>
-        <v>8.7147057000747097E-6</v>
+        <v>6.7514443800106294E-3</v>
       </c>
       <c r="E7" s="46">
         <f t="shared" ca="1" si="0"/>
-        <v>171.91388787794077</v>
+        <v>173.90906022384939</v>
       </c>
       <c r="F7" s="45">
         <f t="shared" ca="1" si="0"/>
@@ -13132,7 +13125,7 @@
       </c>
       <c r="G7" s="45">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>-9.9920072216264089E-16</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -13141,19 +13134,19 @@
       </c>
       <c r="B8" s="47">
         <f t="shared" ref="B8:G8" ca="1" si="1">STDEV(B11:B1010)</f>
-        <v>0.50749596530896357</v>
+        <v>14.169890679628834</v>
       </c>
       <c r="C8" s="45">
         <f t="shared" ca="1" si="1"/>
-        <v>0.50749596530896357</v>
+        <v>14.169890679628834</v>
       </c>
       <c r="D8" s="48">
         <f t="shared" ca="1" si="1"/>
-        <v>5.9041489388633687E-3</v>
+        <v>0.16461148660550934</v>
       </c>
       <c r="E8" s="47">
         <f t="shared" ca="1" si="1"/>
-        <v>1.0149963532959259</v>
+        <v>28.435448588051941</v>
       </c>
       <c r="F8" s="45">
         <f t="shared" ca="1" si="1"/>
@@ -13161,7 +13154,7 @@
       </c>
       <c r="G8" s="45">
         <f t="shared" ca="1" si="1"/>
-        <v>1</v>
+        <v>0.99999999999999989</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -13199,27 +13192,27 @@
       </c>
       <c r="B11" s="50">
         <f ca="1">IF(ISNUMBER(A11),_xlfn.NORM.INV(RAND(),$B$2,$B$3),"")</f>
-        <v>171.55353587356345</v>
+        <v>182.76242262718137</v>
       </c>
       <c r="C11" s="50">
         <f ca="1">IF(ISNUMBER(B11),(SUM($B$11:$B$1010)-B11)/($B$4-1),"")</f>
-        <v>172.27124355055301</v>
+        <v>162.72317105070618</v>
       </c>
       <c r="D11" s="45">
         <f t="shared" ref="D11:D74" ca="1" si="2">IF(ISNUMBER(B11),(($B$4-1)*B11/(SUM($B$11:$B$1010)-B11)-1),"")</f>
-        <v>-4.1661490461055717E-3</v>
+        <v>0.12314934281996481</v>
       </c>
       <c r="E11" s="50">
         <f t="shared" ref="E11:E74" ca="1" si="3">IF(ISNUMBER(B11),AVERAGE($B$11:$B$1010)*(1+D11),"")</f>
-        <v>171.1961770736456</v>
+        <v>194.0159587465424</v>
       </c>
       <c r="F11" s="45">
         <f t="shared" ref="F11:F74" ca="1" si="4">IF(ISNUMBER(D11),(D11-AVERAGE($D$11:$D$1010))/STDEV($D$11:$D$1010),"")</f>
-        <v>-0.70710678118654746</v>
+        <v>0.70710678118654746</v>
       </c>
       <c r="G11" s="45">
         <f t="shared" ref="G11:G74" ca="1" si="5">IF(ISNUMBER(B11),(B11-AVERAGE($B$11:$B$20))/STDEV($B$11:$B$20),"")</f>
-        <v>-0.70710678118654757</v>
+        <v>0.70710678118654646</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -13229,27 +13222,27 @@
       </c>
       <c r="B12" s="50">
         <f t="shared" ref="B12:B75" ca="1" si="6">IF(ISNUMBER(A12),_xlfn.NORM.INV(RAND(),$B$2,$B$3),"")</f>
-        <v>172.27124355055301</v>
+        <v>162.72317105070616</v>
       </c>
       <c r="C12" s="50">
         <f t="shared" ref="C12:C75" ca="1" si="7">IF(ISNUMBER(B12),(SUM($B$11:$B$1010)-B12)/($B$4-1),"")</f>
-        <v>171.55353587356345</v>
+        <v>182.76242262718139</v>
       </c>
       <c r="D12" s="45">
         <f t="shared" ca="1" si="2"/>
-        <v>4.1835784575057211E-3</v>
+        <v>-0.10964645405994355</v>
       </c>
       <c r="E12" s="50">
         <f t="shared" ca="1" si="3"/>
-        <v>172.63159868223593</v>
+        <v>153.80216170115636</v>
       </c>
       <c r="F12" s="45">
         <f t="shared" ca="1" si="4"/>
-        <v>0.70710678118654746</v>
+        <v>-0.70710678118654746</v>
       </c>
       <c r="G12" s="45">
         <f t="shared" ca="1" si="5"/>
-        <v>0.70710678118654757</v>
+        <v>-0.70710678118654846</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
@@ -43236,40 +43229,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="15.6" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="60" t="s">
+      <c r="B1" s="59" t="s">
         <v>107</v>
       </c>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="J1" s="60" t="s">
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="J1" s="59" t="s">
         <v>106</v>
       </c>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
+      <c r="P1" s="59"/>
     </row>
     <row r="2" spans="2:16" ht="15.6" thickTop="1" x14ac:dyDescent="0.35">
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
-      <c r="D2" s="58" t="s">
+      <c r="D2" s="57" t="s">
         <v>90</v>
       </c>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
       <c r="I2" s="5"/>
-      <c r="J2" s="59" t="s">
+      <c r="J2" s="58" t="s">
         <v>95</v>
       </c>
-      <c r="K2" s="59"/>
+      <c r="K2" s="58"/>
       <c r="L2" s="10">
         <v>11.282097222222223</v>
       </c>
@@ -44629,41 +44622,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:17" ht="15.6" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="60" t="s">
+      <c r="B1" s="59" t="s">
         <v>107</v>
       </c>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="J1" s="60" t="s">
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="J1" s="59" t="s">
         <v>106</v>
       </c>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
+      <c r="P1" s="59"/>
+      <c r="Q1" s="59"/>
     </row>
     <row r="2" spans="2:17" ht="15.6" thickTop="1" x14ac:dyDescent="0.35">
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
-      <c r="D2" s="58" t="s">
+      <c r="D2" s="57" t="s">
         <v>90</v>
       </c>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
       <c r="I2" s="5"/>
-      <c r="J2" s="59" t="s">
+      <c r="J2" s="58" t="s">
         <v>95</v>
       </c>
-      <c r="K2" s="59"/>
+      <c r="K2" s="58"/>
       <c r="L2" s="10">
         <v>11.282097222222223</v>
       </c>
@@ -46132,26 +46125,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="297242e2-fbb8-4c67-99ce-cd3528d8cbc6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2b487279-c3ab-426b-b6cf-53277d34fdd2" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100956A0F4035FD3E439A1375AA81288D3D" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="629d0db9554db0b6d69858e5d10e2081">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="297242e2-fbb8-4c67-99ce-cd3528d8cbc6" xmlns:ns3="2b487279-c3ab-426b-b6cf-53277d34fdd2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="10effca0874d89e46752f2faf5212ccb" ns2:_="" ns3:_="">
     <xsd:import namespace="297242e2-fbb8-4c67-99ce-cd3528d8cbc6"/>
@@ -46374,10 +46347,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="297242e2-fbb8-4c67-99ce-cd3528d8cbc6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2b487279-c3ab-426b-b6cf-53277d34fdd2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D65EDFB4-7AB7-4358-93FB-FC0B1840C267}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6277D62E-5E45-4A72-AFF1-71084806AE04}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="297242e2-fbb8-4c67-99ce-cd3528d8cbc6"/>
+    <ds:schemaRef ds:uri="2b487279-c3ab-426b-b6cf-53277d34fdd2"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -46394,20 +46398,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6277D62E-5E45-4A72-AFF1-71084806AE04}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D65EDFB4-7AB7-4358-93FB-FC0B1840C267}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="297242e2-fbb8-4c67-99ce-cd3528d8cbc6"/>
-    <ds:schemaRef ds:uri="2b487279-c3ab-426b-b6cf-53277d34fdd2"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>